<commit_message>
Cumulative updates to project.
</commit_message>
<xml_diff>
--- a/project/outputs_xlsx_solution/prog-loop.1-wide.xlsx
+++ b/project/outputs_xlsx_solution/prog-loop.1-wide.xlsx
@@ -59,13 +59,16 @@
     <t>addi X2, X0, 124</t>
   </si>
   <si>
-    <t>IS/EX</t>
+    <t>EX</t>
   </si>
   <si>
     <t>fld F2, 200(X0)</t>
   </si>
   <si>
-    <t>WB/CT</t>
+    <t>WB</t>
+  </si>
+  <si>
+    <t>CT</t>
   </si>
   <si>
     <t>fld F0, 0(X1)</t>
@@ -80,12 +83,12 @@
     <t>fadd F0, F0, F4</t>
   </si>
   <si>
-    <t>EX</t>
-  </si>
-  <si>
     <t>fsd F0, 0(X2)</t>
   </si>
   <si>
+    <t>IS</t>
+  </si>
+  <si>
     <t>addi X1, X1, -8</t>
   </si>
   <si>
@@ -95,6 +98,12 @@
     <t>bne X1, X0, 12</t>
   </si>
   <si>
+    <t>CDB Stall</t>
+  </si>
+  <si>
+    <t>FU Stall</t>
+  </si>
+  <si>
     <t>[Legend]</t>
   </si>
   <si>
@@ -104,13 +113,34 @@
     <t>Instruction Decode</t>
   </si>
   <si>
-    <t>Add to Issue Queue/Execute (if instruction is ready, it can start executing in the same cycle it is added to issue queue)</t>
-  </si>
-  <si>
-    <t>Execute</t>
-  </si>
-  <si>
-    <t>Write Back/Commit (instruction can be committed on the same cycle it writes back)</t>
+    <t>Add to Issue Queue</t>
+  </si>
+  <si>
+    <t>Execute (instruction can execute on the same cycle as it is added to the issue queue, if it is ready)</t>
+  </si>
+  <si>
+    <t>Write Back</t>
+  </si>
+  <si>
+    <t>Commit (instruction can commit on the same cycle as write back, if at the head)</t>
+  </si>
+  <si>
+    <t>RS Stall</t>
+  </si>
+  <si>
+    <t>Reservation Station Stall (stalled because reservation stations are full)</t>
+  </si>
+  <si>
+    <t>ROB Stall</t>
+  </si>
+  <si>
+    <t>Reorder Buffer Stall (stalled because the ROB is full)</t>
+  </si>
+  <si>
+    <t>Common Data Bus Stall (stalled because the CDB bandwidth is saturated)</t>
+  </si>
+  <si>
+    <t>Functional Unit Stall (stalled because the functional unit is busy)</t>
   </si>
 </sst>
 </file>
@@ -588,6 +618,18 @@
       <c r="AN1">
         <v>37</v>
       </c>
+      <c r="AO1">
+        <v>38</v>
+      </c>
+      <c r="AP1">
+        <v>39</v>
+      </c>
+      <c r="AQ1">
+        <v>40</v>
+      </c>
+      <c r="AR1">
+        <v>41</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -609,7 +651,7 @@
         <v>8</v>
       </c>
       <c r="G2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
@@ -632,7 +674,7 @@
         <v>8</v>
       </c>
       <c r="H3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -655,7 +697,7 @@
         <v>8</v>
       </c>
       <c r="I4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -666,7 +708,7 @@
         <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G5" t="s">
         <v>5</v>
@@ -678,7 +720,7 @@
         <v>8</v>
       </c>
       <c r="J5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -689,7 +731,7 @@
         <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H6" t="s">
         <v>5</v>
@@ -701,16 +743,16 @@
         <v>8</v>
       </c>
       <c r="K6" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="L6" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="M6" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="N6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
@@ -721,7 +763,7 @@
         <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I7" t="s">
         <v>5</v>
@@ -735,8 +777,8 @@
       <c r="L7" t="s">
         <v>10</v>
       </c>
-      <c r="N7" t="s">
-        <v>10</v>
+      <c r="O7" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="8">
@@ -747,7 +789,7 @@
         <v>24</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J8" t="s">
         <v>5</v>
@@ -756,19 +798,19 @@
         <v>6</v>
       </c>
       <c r="L8" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="N8" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="O8" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="P8" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="Q8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
@@ -788,13 +830,13 @@
         <v>6</v>
       </c>
       <c r="M9" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="Q9" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="R9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10">
@@ -805,7 +847,7 @@
         <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="L10" t="s">
         <v>5</v>
@@ -819,8 +861,8 @@
       <c r="O10" t="s">
         <v>10</v>
       </c>
-      <c r="R10" t="s">
-        <v>10</v>
+      <c r="S10" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -831,7 +873,7 @@
         <v>36</v>
       </c>
       <c r="C11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M11" t="s">
         <v>5</v>
@@ -845,8 +887,8 @@
       <c r="P11" t="s">
         <v>10</v>
       </c>
-      <c r="R11" t="s">
-        <v>10</v>
+      <c r="T11" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="12">
@@ -857,7 +899,7 @@
         <v>40</v>
       </c>
       <c r="C12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="N12" t="s">
         <v>5</v>
@@ -866,13 +908,16 @@
         <v>6</v>
       </c>
       <c r="P12" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="Q12" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="R12" t="s">
         <v>10</v>
+      </c>
+      <c r="U12" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="13">
@@ -883,7 +928,7 @@
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R13" t="s">
         <v>5</v>
@@ -896,6 +941,9 @@
       </c>
       <c r="U13" t="s">
         <v>10</v>
+      </c>
+      <c r="V13" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="14">
@@ -906,7 +954,7 @@
         <v>16</v>
       </c>
       <c r="C14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S14" t="s">
         <v>5</v>
@@ -915,19 +963,28 @@
         <v>6</v>
       </c>
       <c r="U14" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="V14" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="W14" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="X14" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="Y14" t="s">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>21</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>21</v>
+      </c>
+      <c r="AB14" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="15">
@@ -938,7 +995,7 @@
         <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T15" t="s">
         <v>5</v>
@@ -952,8 +1009,8 @@
       <c r="W15" t="s">
         <v>10</v>
       </c>
-      <c r="Y15" t="s">
-        <v>10</v>
+      <c r="AC15" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="16">
@@ -964,7 +1021,7 @@
         <v>24</v>
       </c>
       <c r="C16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="U16" t="s">
         <v>5</v>
@@ -973,19 +1030,19 @@
         <v>6</v>
       </c>
       <c r="W16" t="s">
-        <v>8</v>
-      </c>
-      <c r="Y16" t="s">
-        <v>15</v>
-      </c>
-      <c r="Z16" t="s">
-        <v>15</v>
-      </c>
-      <c r="AA16" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="AB16" t="s">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>8</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>8</v>
+      </c>
+      <c r="AE16" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="17">
@@ -1005,13 +1062,16 @@
         <v>6</v>
       </c>
       <c r="X17" t="s">
-        <v>8</v>
-      </c>
-      <c r="AB17" t="s">
-        <v>15</v>
-      </c>
-      <c r="AC17" t="s">
-        <v>10</v>
+        <v>17</v>
+      </c>
+      <c r="AE17" t="s">
+        <v>22</v>
+      </c>
+      <c r="AF17" t="s">
+        <v>8</v>
+      </c>
+      <c r="AG17" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="18">
@@ -1022,7 +1082,7 @@
         <v>32</v>
       </c>
       <c r="C18" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="W18" t="s">
         <v>5</v>
@@ -1036,8 +1096,8 @@
       <c r="Z18" t="s">
         <v>10</v>
       </c>
-      <c r="AC18" t="s">
-        <v>10</v>
+      <c r="AH18" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="19">
@@ -1048,7 +1108,7 @@
         <v>36</v>
       </c>
       <c r="C19" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X19" t="s">
         <v>5</v>
@@ -1062,202 +1122,217 @@
       <c r="AA19" t="s">
         <v>10</v>
       </c>
-      <c r="AC19" t="s">
-        <v>10</v>
+      <c r="AI19" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="20">
       <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>40</v>
+      </c>
+      <c r="C20" t="s">
         <v>20</v>
       </c>
-      <c r="B20">
-        <v>12</v>
-      </c>
-      <c r="C20" t="s">
-        <v>11</v>
+      <c r="Y20" t="s">
+        <v>5</v>
       </c>
       <c r="Z20" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA20" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="AB20" t="s">
         <v>8</v>
       </c>
       <c r="AC20" t="s">
-        <v>15</v>
-      </c>
-      <c r="AD20" t="s">
-        <v>10</v>
+        <v>10</v>
+      </c>
+      <c r="AJ20" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="21">
       <c r="A21">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C21" t="s">
         <v>12</v>
       </c>
+      <c r="Z21" t="s">
+        <v>5</v>
+      </c>
       <c r="AA21" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AB21" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="AC21" t="s">
         <v>8</v>
       </c>
       <c r="AD21" t="s">
-        <v>15</v>
-      </c>
-      <c r="AE21" t="s">
-        <v>15</v>
-      </c>
-      <c r="AF21" t="s">
-        <v>15</v>
-      </c>
-      <c r="AG21" t="s">
-        <v>15</v>
-      </c>
-      <c r="AH21" t="s">
-        <v>15</v>
-      </c>
-      <c r="AI21" t="s">
-        <v>15</v>
-      </c>
-      <c r="AJ21" t="s">
-        <v>10</v>
+        <v>10</v>
+      </c>
+      <c r="AK21" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="22">
       <c r="A22">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B22">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C22" t="s">
         <v>13</v>
       </c>
+      <c r="AA22" t="s">
+        <v>5</v>
+      </c>
       <c r="AB22" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AC22" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="AD22" t="s">
         <v>8</v>
       </c>
       <c r="AE22" t="s">
-        <v>10</v>
-      </c>
-      <c r="AJ22" t="s">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="AF22" t="s">
+        <v>8</v>
+      </c>
+      <c r="AG22" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH22" t="s">
+        <v>10</v>
+      </c>
+      <c r="AL22" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="23">
       <c r="A23">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B23">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C23" t="s">
         <v>14</v>
       </c>
+      <c r="AB23" t="s">
+        <v>5</v>
+      </c>
       <c r="AC23" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AD23" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="AE23" t="s">
         <v>8</v>
       </c>
-      <c r="AJ23" t="s">
-        <v>15</v>
-      </c>
-      <c r="AK23" t="s">
-        <v>15</v>
-      </c>
-      <c r="AL23" t="s">
-        <v>15</v>
+      <c r="AF23" t="s">
+        <v>10</v>
       </c>
       <c r="AM23" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24">
       <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24">
         <v>24</v>
       </c>
-      <c r="B24">
-        <v>28</v>
-      </c>
       <c r="C24" t="s">
-        <v>16</v>
+        <v>15</v>
+      </c>
+      <c r="AC24" t="s">
+        <v>5</v>
       </c>
       <c r="AD24" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AE24" t="s">
-        <v>6</v>
-      </c>
-      <c r="AF24" t="s">
-        <v>8</v>
-      </c>
-      <c r="AM24" t="s">
-        <v>15</v>
+        <v>17</v>
+      </c>
+      <c r="AH24" t="s">
+        <v>8</v>
+      </c>
+      <c r="AI24" t="s">
+        <v>8</v>
+      </c>
+      <c r="AJ24" t="s">
+        <v>8</v>
+      </c>
+      <c r="AK24" t="s">
+        <v>10</v>
       </c>
       <c r="AN24" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25">
       <c r="A25">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C25" t="s">
-        <v>17</v>
+        <v>16</v>
+      </c>
+      <c r="AD25" t="s">
+        <v>5</v>
       </c>
       <c r="AE25" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AF25" t="s">
-        <v>6</v>
-      </c>
-      <c r="AG25" t="s">
-        <v>8</v>
-      </c>
-      <c r="AH25" t="s">
-        <v>10</v>
-      </c>
-      <c r="AN25" t="s">
-        <v>10</v>
+        <v>17</v>
+      </c>
+      <c r="AK25" t="s">
+        <v>8</v>
+      </c>
+      <c r="AL25" t="s">
+        <v>10</v>
+      </c>
+      <c r="AO25" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="26">
       <c r="A26">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B26">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C26" t="s">
         <v>18</v>
       </c>
+      <c r="AE26" t="s">
+        <v>5</v>
+      </c>
       <c r="AF26" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG26" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="AH26" t="s">
         <v>8</v>
@@ -1265,82 +1340,151 @@
       <c r="AI26" t="s">
         <v>10</v>
       </c>
-      <c r="AN26" t="s">
-        <v>10</v>
+      <c r="AP26" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="27">
       <c r="A27">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B27">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C27" t="s">
         <v>19</v>
       </c>
+      <c r="AF27" t="s">
+        <v>5</v>
+      </c>
       <c r="AG27" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH27" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="AI27" t="s">
         <v>8</v>
       </c>
       <c r="AJ27" t="s">
-        <v>15</v>
-      </c>
-      <c r="AK27" t="s">
-        <v>10</v>
-      </c>
-      <c r="AN27" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="s">
+        <v>10</v>
+      </c>
+      <c r="AQ27" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>40</v>
+      </c>
+      <c r="C28" t="s">
         <v>20</v>
+      </c>
+      <c r="AG28" t="s">
+        <v>5</v>
+      </c>
+      <c r="AH28" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI28" t="s">
+        <v>17</v>
+      </c>
+      <c r="AJ28" t="s">
+        <v>8</v>
+      </c>
+      <c r="AK28" t="s">
+        <v>10</v>
+      </c>
+      <c r="AR28" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>5</v>
-      </c>
-      <c r="B30" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B31" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B32" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B33" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B34" t="s">
-        <v>25</v>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>10</v>
+      </c>
+      <c r="B35" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>11</v>
+      </c>
+      <c r="B36" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>30</v>
+      </c>
+      <c r="B37" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>32</v>
+      </c>
+      <c r="B38" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>21</v>
+      </c>
+      <c r="B39" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>22</v>
+      </c>
+      <c r="B40" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed bug where instructions were not getting immediately issued even when the operands are ready, if the operands had not been committed, resulting in an extra "IS" stage before the "EX" stage.
</commit_message>
<xml_diff>
--- a/project/outputs_xlsx_solution/prog-loop.1-wide.xlsx
+++ b/project/outputs_xlsx_solution/prog-loop.1-wide.xlsx
@@ -98,10 +98,10 @@
     <t>bne X1, X0, 12</t>
   </si>
   <si>
+    <t>FU Stall</t>
+  </si>
+  <si>
     <t>CDB Stall</t>
-  </si>
-  <si>
-    <t>FU Stall</t>
   </si>
   <si>
     <t>[Legend]</t>
@@ -624,12 +624,6 @@
       <c r="AP1">
         <v>39</v>
       </c>
-      <c r="AQ1">
-        <v>40</v>
-      </c>
-      <c r="AR1">
-        <v>41</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -908,12 +902,9 @@
         <v>6</v>
       </c>
       <c r="P12" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="Q12" t="s">
-        <v>8</v>
-      </c>
-      <c r="R12" t="s">
         <v>10</v>
       </c>
       <c r="U12" t="s">
@@ -930,16 +921,16 @@
       <c r="C13" t="s">
         <v>12</v>
       </c>
+      <c r="Q13" t="s">
+        <v>5</v>
+      </c>
       <c r="R13" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S13" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="T13" t="s">
-        <v>8</v>
-      </c>
-      <c r="U13" t="s">
         <v>10</v>
       </c>
       <c r="V13" t="s">
@@ -956,14 +947,17 @@
       <c r="C14" t="s">
         <v>13</v>
       </c>
+      <c r="R14" t="s">
+        <v>5</v>
+      </c>
       <c r="S14" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T14" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U14" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="V14" t="s">
         <v>8</v>
@@ -972,18 +966,6 @@
         <v>8</v>
       </c>
       <c r="X14" t="s">
-        <v>8</v>
-      </c>
-      <c r="Y14" t="s">
-        <v>8</v>
-      </c>
-      <c r="Z14" t="s">
-        <v>21</v>
-      </c>
-      <c r="AA14" t="s">
-        <v>21</v>
-      </c>
-      <c r="AB14" t="s">
         <v>11</v>
       </c>
     </row>
@@ -997,19 +979,19 @@
       <c r="C15" t="s">
         <v>14</v>
       </c>
+      <c r="S15" t="s">
+        <v>5</v>
+      </c>
       <c r="T15" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U15" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V15" t="s">
-        <v>8</v>
-      </c>
-      <c r="W15" t="s">
-        <v>10</v>
-      </c>
-      <c r="AC15" t="s">
+        <v>10</v>
+      </c>
+      <c r="Y15" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1023,25 +1005,25 @@
       <c r="C16" t="s">
         <v>15</v>
       </c>
+      <c r="T16" t="s">
+        <v>5</v>
+      </c>
       <c r="U16" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V16" t="s">
-        <v>6</v>
-      </c>
-      <c r="W16" t="s">
         <v>17</v>
       </c>
-      <c r="AB16" t="s">
-        <v>8</v>
-      </c>
-      <c r="AC16" t="s">
-        <v>8</v>
-      </c>
-      <c r="AD16" t="s">
-        <v>8</v>
-      </c>
-      <c r="AE16" t="s">
+      <c r="X16" t="s">
+        <v>8</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>8</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA16" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1055,22 +1037,19 @@
       <c r="C17" t="s">
         <v>16</v>
       </c>
+      <c r="U17" t="s">
+        <v>5</v>
+      </c>
       <c r="V17" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W17" t="s">
-        <v>6</v>
-      </c>
-      <c r="X17" t="s">
         <v>17</v>
       </c>
-      <c r="AE17" t="s">
-        <v>22</v>
-      </c>
-      <c r="AF17" t="s">
-        <v>8</v>
-      </c>
-      <c r="AG17" t="s">
+      <c r="AA17" t="s">
+        <v>8</v>
+      </c>
+      <c r="AB17" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1084,19 +1063,19 @@
       <c r="C18" t="s">
         <v>18</v>
       </c>
+      <c r="V18" t="s">
+        <v>5</v>
+      </c>
       <c r="W18" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X18" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Y18" t="s">
-        <v>8</v>
-      </c>
-      <c r="Z18" t="s">
-        <v>10</v>
-      </c>
-      <c r="AH18" t="s">
+        <v>10</v>
+      </c>
+      <c r="AC18" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1110,19 +1089,19 @@
       <c r="C19" t="s">
         <v>19</v>
       </c>
+      <c r="W19" t="s">
+        <v>5</v>
+      </c>
       <c r="X19" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y19" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Z19" t="s">
-        <v>8</v>
-      </c>
-      <c r="AA19" t="s">
-        <v>10</v>
-      </c>
-      <c r="AI19" t="s">
+        <v>10</v>
+      </c>
+      <c r="AD19" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1136,22 +1115,19 @@
       <c r="C20" t="s">
         <v>20</v>
       </c>
+      <c r="X20" t="s">
+        <v>5</v>
+      </c>
       <c r="Y20" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Z20" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AA20" t="s">
-        <v>17</v>
-      </c>
-      <c r="AB20" t="s">
-        <v>8</v>
-      </c>
-      <c r="AC20" t="s">
-        <v>10</v>
-      </c>
-      <c r="AJ20" t="s">
+        <v>10</v>
+      </c>
+      <c r="AE20" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1165,22 +1141,22 @@
       <c r="C21" t="s">
         <v>12</v>
       </c>
+      <c r="Y21" t="s">
+        <v>5</v>
+      </c>
       <c r="Z21" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA21" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="AB21" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="AC21" t="s">
-        <v>8</v>
-      </c>
-      <c r="AD21" t="s">
-        <v>10</v>
-      </c>
-      <c r="AK21" t="s">
+        <v>10</v>
+      </c>
+      <c r="AF21" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1194,14 +1170,17 @@
       <c r="C22" t="s">
         <v>13</v>
       </c>
+      <c r="Z22" t="s">
+        <v>5</v>
+      </c>
       <c r="AA22" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AB22" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="AC22" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="AD22" t="s">
         <v>8</v>
@@ -1213,12 +1192,12 @@
         <v>8</v>
       </c>
       <c r="AG22" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="AH22" t="s">
-        <v>10</v>
-      </c>
-      <c r="AL22" t="s">
+        <v>22</v>
+      </c>
+      <c r="AI22" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1232,22 +1211,19 @@
       <c r="C23" t="s">
         <v>14</v>
       </c>
+      <c r="AA23" t="s">
+        <v>5</v>
+      </c>
       <c r="AB23" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AC23" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AD23" t="s">
-        <v>17</v>
-      </c>
-      <c r="AE23" t="s">
-        <v>8</v>
-      </c>
-      <c r="AF23" t="s">
-        <v>10</v>
-      </c>
-      <c r="AM23" t="s">
+        <v>10</v>
+      </c>
+      <c r="AJ23" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1261,18 +1237,15 @@
       <c r="C24" t="s">
         <v>15</v>
       </c>
+      <c r="AB24" t="s">
+        <v>5</v>
+      </c>
       <c r="AC24" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AD24" t="s">
-        <v>6</v>
-      </c>
-      <c r="AE24" t="s">
         <v>17</v>
       </c>
-      <c r="AH24" t="s">
-        <v>8</v>
-      </c>
       <c r="AI24" t="s">
         <v>8</v>
       </c>
@@ -1280,9 +1253,9 @@
         <v>8</v>
       </c>
       <c r="AK24" t="s">
-        <v>10</v>
-      </c>
-      <c r="AN24" t="s">
+        <v>8</v>
+      </c>
+      <c r="AL24" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1296,22 +1269,19 @@
       <c r="C25" t="s">
         <v>16</v>
       </c>
+      <c r="AC25" t="s">
+        <v>5</v>
+      </c>
       <c r="AD25" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AE25" t="s">
-        <v>6</v>
-      </c>
-      <c r="AF25" t="s">
         <v>17</v>
       </c>
-      <c r="AK25" t="s">
-        <v>8</v>
-      </c>
       <c r="AL25" t="s">
-        <v>10</v>
-      </c>
-      <c r="AO25" t="s">
+        <v>8</v>
+      </c>
+      <c r="AM25" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1325,22 +1295,19 @@
       <c r="C26" t="s">
         <v>18</v>
       </c>
+      <c r="AD26" t="s">
+        <v>5</v>
+      </c>
       <c r="AE26" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AF26" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AG26" t="s">
-        <v>17</v>
-      </c>
-      <c r="AH26" t="s">
-        <v>8</v>
-      </c>
-      <c r="AI26" t="s">
-        <v>10</v>
-      </c>
-      <c r="AP26" t="s">
+        <v>10</v>
+      </c>
+      <c r="AN26" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1354,22 +1321,19 @@
       <c r="C27" t="s">
         <v>19</v>
       </c>
+      <c r="AE27" t="s">
+        <v>5</v>
+      </c>
       <c r="AF27" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG27" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AH27" t="s">
-        <v>17</v>
-      </c>
-      <c r="AI27" t="s">
-        <v>8</v>
-      </c>
-      <c r="AJ27" t="s">
-        <v>10</v>
-      </c>
-      <c r="AQ27" t="s">
+        <v>10</v>
+      </c>
+      <c r="AO27" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1383,22 +1347,19 @@
       <c r="C28" t="s">
         <v>20</v>
       </c>
+      <c r="AF28" t="s">
+        <v>5</v>
+      </c>
       <c r="AG28" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH28" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AI28" t="s">
-        <v>17</v>
-      </c>
-      <c r="AJ28" t="s">
-        <v>8</v>
-      </c>
-      <c r="AK28" t="s">
-        <v>10</v>
-      </c>
-      <c r="AR28" t="s">
+        <v>10</v>
+      </c>
+      <c r="AP28" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1473,7 +1434,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B39" t="s">
         <v>34</v>
@@ -1481,7 +1442,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B40" t="s">
         <v>35</v>

</xml_diff>